<commit_message>
revision files submitted to GC
</commit_message>
<xml_diff>
--- a/Scripts/Prices regionalization.xlsx
+++ b/Scripts/Prices regionalization.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\anabera\Desktop\Fossil vs. green chemicals\Scripts\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{6738AC1D-DBF8-434C-9A0C-775775C9AA5B}" xr6:coauthVersionLast="36" xr6:coauthVersionMax="36" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{562D5297-5F84-427C-B858-9769622F51DE}" xr6:coauthVersionLast="36" xr6:coauthVersionMax="36" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="0" windowWidth="17280" windowHeight="8088" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="0" yWindow="0" windowWidth="17280" windowHeight="8088" firstSheet="3" activeTab="12" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Wind LCOH countries" sheetId="1" r:id="rId1"/>
@@ -37,7 +37,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="631" uniqueCount="83">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="634" uniqueCount="86">
   <si>
     <t>Country</t>
   </si>
@@ -287,6 +287,15 @@
   <si>
     <t>Both inflation and natural gas</t>
   </si>
+  <si>
+    <t>PPP</t>
+  </si>
+  <si>
+    <t>Exchange rates</t>
+  </si>
+  <si>
+    <t>PPP in LCU</t>
+  </si>
 </sst>
 </file>
 
@@ -365,7 +374,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="41">
+  <cellXfs count="42">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="center"/>
@@ -458,6 +467,9 @@
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="1" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
@@ -561,7 +573,7 @@
               <a:cs typeface="+mn-cs"/>
             </a:defRPr>
           </a:pPr>
-          <a:endParaRPr lang="de-DE"/>
+          <a:endParaRPr lang="en-US"/>
         </a:p>
       </c:txPr>
     </c:title>
@@ -913,7 +925,7 @@
                 <a:cs typeface="+mn-cs"/>
               </a:defRPr>
             </a:pPr>
-            <a:endParaRPr lang="de-DE"/>
+            <a:endParaRPr lang="en-US"/>
           </a:p>
         </c:txPr>
         <c:crossAx val="1589179247"/>
@@ -1012,7 +1024,7 @@
                   <a:cs typeface="+mn-cs"/>
                 </a:defRPr>
               </a:pPr>
-              <a:endParaRPr lang="de-DE"/>
+              <a:endParaRPr lang="en-US"/>
             </a:p>
           </c:txPr>
         </c:title>
@@ -1046,7 +1058,7 @@
                 <a:cs typeface="+mn-cs"/>
               </a:defRPr>
             </a:pPr>
-            <a:endParaRPr lang="de-DE"/>
+            <a:endParaRPr lang="en-US"/>
           </a:p>
         </c:txPr>
         <c:crossAx val="1643752831"/>
@@ -1088,7 +1100,7 @@
               <a:cs typeface="+mn-cs"/>
             </a:defRPr>
           </a:pPr>
-          <a:endParaRPr lang="de-DE"/>
+          <a:endParaRPr lang="en-US"/>
         </a:p>
       </c:txPr>
     </c:legend>
@@ -1118,7 +1130,7 @@
       <a:pPr>
         <a:defRPr/>
       </a:pPr>
-      <a:endParaRPr lang="de-DE"/>
+      <a:endParaRPr lang="en-US"/>
     </a:p>
   </c:txPr>
   <c:printSettings>
@@ -1194,7 +1206,7 @@
               <a:cs typeface="+mn-cs"/>
             </a:defRPr>
           </a:pPr>
-          <a:endParaRPr lang="de-DE"/>
+          <a:endParaRPr lang="en-US"/>
         </a:p>
       </c:txPr>
     </c:title>
@@ -1546,7 +1558,7 @@
                 <a:cs typeface="+mn-cs"/>
               </a:defRPr>
             </a:pPr>
-            <a:endParaRPr lang="de-DE"/>
+            <a:endParaRPr lang="en-US"/>
           </a:p>
         </c:txPr>
         <c:crossAx val="1589179247"/>
@@ -1645,7 +1657,7 @@
                   <a:cs typeface="+mn-cs"/>
                 </a:defRPr>
               </a:pPr>
-              <a:endParaRPr lang="de-DE"/>
+              <a:endParaRPr lang="en-US"/>
             </a:p>
           </c:txPr>
         </c:title>
@@ -1679,7 +1691,7 @@
                 <a:cs typeface="+mn-cs"/>
               </a:defRPr>
             </a:pPr>
-            <a:endParaRPr lang="de-DE"/>
+            <a:endParaRPr lang="en-US"/>
           </a:p>
         </c:txPr>
         <c:crossAx val="1643752831"/>
@@ -1721,7 +1733,7 @@
               <a:cs typeface="+mn-cs"/>
             </a:defRPr>
           </a:pPr>
-          <a:endParaRPr lang="de-DE"/>
+          <a:endParaRPr lang="en-US"/>
         </a:p>
       </c:txPr>
     </c:legend>
@@ -1746,7 +1758,7 @@
       <a:pPr>
         <a:defRPr/>
       </a:pPr>
-      <a:endParaRPr lang="de-DE"/>
+      <a:endParaRPr lang="en-US"/>
     </a:p>
   </c:txPr>
   <c:printSettings>
@@ -3262,21 +3274,21 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:24" x14ac:dyDescent="0.3">
-      <c r="B1" s="34">
+      <c r="B1" s="35">
         <v>2019</v>
       </c>
-      <c r="C1" s="34"/>
-      <c r="D1" s="34"/>
-      <c r="E1" s="34">
+      <c r="C1" s="35"/>
+      <c r="D1" s="35"/>
+      <c r="E1" s="35">
         <v>2020</v>
       </c>
-      <c r="F1" s="34"/>
-      <c r="G1" s="34"/>
-      <c r="H1" s="34">
+      <c r="F1" s="35"/>
+      <c r="G1" s="35"/>
+      <c r="H1" s="35">
         <v>2021</v>
       </c>
-      <c r="I1" s="34"/>
-      <c r="J1" s="34"/>
+      <c r="I1" s="35"/>
+      <c r="J1" s="35"/>
       <c r="K1" s="2">
         <v>2022</v>
       </c>
@@ -11940,15 +11952,16 @@
 
 <file path=xl/worksheets/sheet13.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{4D099D41-EC54-4A9B-8F6F-871BB4D178AD}">
-  <dimension ref="A1:K17"/>
+  <dimension ref="A1:L17"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="2" max="8" width="9.5546875" bestFit="1" customWidth="1"/>
     <col min="9" max="9" width="11" bestFit="1" customWidth="1"/>
     <col min="10" max="11" width="9.5546875" bestFit="1" customWidth="1"/>
+    <col min="12" max="12" width="13.33203125" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:11" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A1" s="19" t="s">
         <v>78</v>
       </c>
@@ -11982,8 +11995,11 @@
       <c r="K1" s="19" t="s">
         <v>77</v>
       </c>
-    </row>
-    <row r="2" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="L1" s="34" t="s">
+        <v>85</v>
+      </c>
+    </row>
+    <row r="2" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A2" s="19">
         <v>2019</v>
       </c>
@@ -12019,7 +12035,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="3" spans="1:11" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A3" s="19">
         <v>2020</v>
       </c>
@@ -12054,7 +12070,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="4" spans="1:11" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A4" s="19">
         <v>2021</v>
       </c>
@@ -12089,7 +12105,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="5" spans="1:11" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A5" s="19">
         <v>2022</v>
       </c>
@@ -12124,7 +12140,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="7" spans="1:11" x14ac:dyDescent="0.3">
+    <row r="7" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A7" s="19" t="s">
         <v>78</v>
       </c>
@@ -12158,8 +12174,11 @@
       <c r="K7" s="19" t="s">
         <v>77</v>
       </c>
-    </row>
-    <row r="8" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="L7" s="34" t="s">
+        <v>84</v>
+      </c>
+    </row>
+    <row r="8" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A8" s="19">
         <v>2019</v>
       </c>
@@ -12194,7 +12213,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="9" spans="1:11" x14ac:dyDescent="0.3">
+    <row r="9" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A9" s="19">
         <v>2020</v>
       </c>
@@ -12229,7 +12248,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="10" spans="1:11" x14ac:dyDescent="0.3">
+    <row r="10" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A10" s="19">
         <v>2021</v>
       </c>
@@ -12264,7 +12283,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="11" spans="1:11" x14ac:dyDescent="0.3">
+    <row r="11" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A11" s="19">
         <v>2022</v>
       </c>
@@ -12299,7 +12318,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="12" spans="1:11" x14ac:dyDescent="0.3">
+    <row r="12" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A12" s="19"/>
       <c r="B12" s="20"/>
       <c r="C12" s="20"/>
@@ -12312,7 +12331,7 @@
       <c r="J12" s="20"/>
       <c r="K12" s="20"/>
     </row>
-    <row r="13" spans="1:11" x14ac:dyDescent="0.3">
+    <row r="13" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A13" s="19" t="s">
         <v>79</v>
       </c>
@@ -12346,8 +12365,11 @@
       <c r="K13" s="19" t="s">
         <v>77</v>
       </c>
-    </row>
-    <row r="14" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="L13" s="34" t="s">
+        <v>83</v>
+      </c>
+    </row>
+    <row r="14" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A14" s="19">
         <v>2019</v>
       </c>
@@ -12392,7 +12414,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="15" spans="1:11" x14ac:dyDescent="0.3">
+    <row r="15" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A15" s="19">
         <v>2020</v>
       </c>
@@ -12437,7 +12459,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="16" spans="1:11" x14ac:dyDescent="0.3">
+    <row r="16" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A16" s="19">
         <v>2021</v>
       </c>
@@ -12545,21 +12567,21 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:22" x14ac:dyDescent="0.3">
-      <c r="B1" s="34">
+      <c r="B1" s="35">
         <v>2019</v>
       </c>
-      <c r="C1" s="34"/>
-      <c r="D1" s="34"/>
-      <c r="E1" s="34">
+      <c r="C1" s="35"/>
+      <c r="D1" s="35"/>
+      <c r="E1" s="35">
         <v>2020</v>
       </c>
-      <c r="F1" s="34"/>
-      <c r="G1" s="34"/>
-      <c r="H1" s="34">
+      <c r="F1" s="35"/>
+      <c r="G1" s="35"/>
+      <c r="H1" s="35">
         <v>2021</v>
       </c>
-      <c r="I1" s="34"/>
-      <c r="J1" s="34"/>
+      <c r="I1" s="35"/>
+      <c r="J1" s="35"/>
       <c r="K1" s="10">
         <v>2022</v>
       </c>
@@ -13219,7 +13241,7 @@
       <c r="I2" s="26">
         <v>6.0595152292610779</v>
       </c>
-      <c r="J2" s="38" t="s">
+      <c r="J2" s="39" t="s">
         <v>80</v>
       </c>
     </row>
@@ -13251,7 +13273,7 @@
       <c r="I3" s="26">
         <v>6.073570022608787</v>
       </c>
-      <c r="J3" s="38"/>
+      <c r="J3" s="39"/>
     </row>
     <row r="4" spans="1:18" x14ac:dyDescent="0.3">
       <c r="A4" s="25" t="s">
@@ -13281,7 +13303,7 @@
       <c r="I4" s="26">
         <v>6.0840794626795969</v>
       </c>
-      <c r="J4" s="38"/>
+      <c r="J4" s="39"/>
     </row>
     <row r="5" spans="1:18" x14ac:dyDescent="0.3">
       <c r="A5" s="25" t="s">
@@ -13311,7 +13333,7 @@
       <c r="I5" s="26">
         <v>6.113455246973909</v>
       </c>
-      <c r="J5" s="38"/>
+      <c r="J5" s="39"/>
     </row>
     <row r="6" spans="1:18" x14ac:dyDescent="0.3">
       <c r="A6" s="25" t="s">
@@ -13341,7 +13363,7 @@
       <c r="I6" s="26">
         <v>6.1535683869068301</v>
       </c>
-      <c r="J6" s="38"/>
+      <c r="J6" s="39"/>
     </row>
     <row r="7" spans="1:18" x14ac:dyDescent="0.3">
       <c r="A7" s="25" t="s">
@@ -13371,7 +13393,7 @@
       <c r="I7" s="26">
         <v>6.1822097765937842</v>
       </c>
-      <c r="J7" s="38"/>
+      <c r="J7" s="39"/>
     </row>
     <row r="8" spans="1:18" x14ac:dyDescent="0.3">
       <c r="A8" s="25" t="s">
@@ -13401,7 +13423,7 @@
       <c r="I8" s="26">
         <v>6.1996290378471226</v>
       </c>
-      <c r="J8" s="38"/>
+      <c r="J8" s="39"/>
     </row>
     <row r="9" spans="1:18" x14ac:dyDescent="0.3">
       <c r="A9" s="25" t="s">
@@ -13431,7 +13453,7 @@
       <c r="I9" s="26">
         <v>6.2076603483315287</v>
       </c>
-      <c r="J9" s="38"/>
+      <c r="J9" s="39"/>
     </row>
     <row r="10" spans="1:18" x14ac:dyDescent="0.3">
       <c r="A10" s="25" t="s">
@@ -13461,7 +13483,7 @@
       <c r="I10" s="26">
         <v>6.2112057016084279</v>
       </c>
-      <c r="J10" s="38"/>
+      <c r="J10" s="39"/>
     </row>
     <row r="11" spans="1:18" x14ac:dyDescent="0.3">
       <c r="A11" s="25" t="s">
@@ -13491,7 +13513,7 @@
       <c r="I11" s="26">
         <v>6.2101674195773358</v>
       </c>
-      <c r="J11" s="38"/>
+      <c r="J11" s="39"/>
     </row>
     <row r="12" spans="1:18" x14ac:dyDescent="0.3">
       <c r="A12" s="23" t="s">
@@ -13521,7 +13543,7 @@
       <c r="I12" s="24">
         <v>6.2082128709201356</v>
       </c>
-      <c r="J12" s="39"/>
+      <c r="J12" s="40"/>
     </row>
     <row r="13" spans="1:18" x14ac:dyDescent="0.3">
       <c r="A13" s="27" t="s">
@@ -13551,7 +13573,7 @@
       <c r="I13" s="28">
         <v>5.4740716409665193</v>
       </c>
-      <c r="J13" s="40" t="s">
+      <c r="J13" s="41" t="s">
         <v>81</v>
       </c>
     </row>
@@ -13583,7 +13605,7 @@
       <c r="I14" s="26">
         <v>5.4744347252575922</v>
       </c>
-      <c r="J14" s="38"/>
+      <c r="J14" s="39"/>
     </row>
     <row r="15" spans="1:18" x14ac:dyDescent="0.3">
       <c r="A15" s="25" t="s">
@@ -13613,7 +13635,7 @@
       <c r="I15" s="26">
         <v>5.5433753550250042</v>
       </c>
-      <c r="J15" s="38"/>
+      <c r="J15" s="39"/>
     </row>
     <row r="16" spans="1:18" x14ac:dyDescent="0.3">
       <c r="A16" s="25" t="s">
@@ -13643,7 +13665,7 @@
       <c r="I16" s="26">
         <v>5.4924981687384546</v>
       </c>
-      <c r="J16" s="38"/>
+      <c r="J16" s="39"/>
     </row>
     <row r="17" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A17" s="25" t="s">
@@ -13673,7 +13695,7 @@
       <c r="I17" s="26">
         <v>5.4707584968104817</v>
       </c>
-      <c r="J17" s="38"/>
+      <c r="J17" s="39"/>
     </row>
     <row r="18" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A18" s="25" t="s">
@@ -13703,7 +13725,7 @@
       <c r="I18" s="26">
         <v>5.4843741577257044</v>
       </c>
-      <c r="J18" s="38"/>
+      <c r="J18" s="39"/>
     </row>
     <row r="19" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A19" s="25" t="s">
@@ -13733,7 +13755,7 @@
       <c r="I19" s="26">
         <v>5.5549940523393273</v>
       </c>
-      <c r="J19" s="38"/>
+      <c r="J19" s="39"/>
     </row>
     <row r="20" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A20" s="25" t="s">
@@ -13763,7 +13785,7 @@
       <c r="I20" s="26">
         <v>5.6266578142897838</v>
       </c>
-      <c r="J20" s="38"/>
+      <c r="J20" s="39"/>
     </row>
     <row r="21" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A21" s="25" t="s">
@@ -13793,7 +13815,7 @@
       <c r="I21" s="26">
         <v>5.5433753550250042</v>
       </c>
-      <c r="J21" s="38"/>
+      <c r="J21" s="39"/>
     </row>
     <row r="22" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A22" s="25" t="s">
@@ -13823,7 +13845,7 @@
       <c r="I22" s="26">
         <v>5.4149796725944519</v>
       </c>
-      <c r="J22" s="38"/>
+      <c r="J22" s="39"/>
     </row>
     <row r="23" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A23" s="23" t="s">
@@ -13853,7 +13875,7 @@
       <c r="I23" s="24">
         <v>5.415569684567445</v>
       </c>
-      <c r="J23" s="39"/>
+      <c r="J23" s="40"/>
     </row>
     <row r="24" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A24" s="27" t="s">
@@ -13883,7 +13905,7 @@
       <c r="I24" s="28">
         <v>6.150603795651552</v>
       </c>
-      <c r="J24" s="35" t="s">
+      <c r="J24" s="36" t="s">
         <v>82</v>
       </c>
     </row>
@@ -13915,7 +13937,7 @@
       <c r="I25" s="26">
         <v>6.1655861719250762</v>
       </c>
-      <c r="J25" s="36"/>
+      <c r="J25" s="37"/>
     </row>
     <row r="26" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A26" s="25" t="s">
@@ -13945,7 +13967,7 @@
       <c r="I26" s="26">
         <v>6.2449994696495681</v>
       </c>
-      <c r="J26" s="36"/>
+      <c r="J26" s="37"/>
     </row>
     <row r="27" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A27" s="25" t="s">
@@ -13975,7 +13997,7 @@
       <c r="I27" s="26">
         <v>6.2227138423414967</v>
       </c>
-      <c r="J27" s="36"/>
+      <c r="J27" s="37"/>
     </row>
     <row r="28" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A28" s="25" t="s">
@@ -14005,7 +14027,7 @@
       <c r="I28" s="26">
         <v>6.2396947384975237</v>
       </c>
-      <c r="J28" s="36"/>
+      <c r="J28" s="37"/>
     </row>
     <row r="29" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A29" s="25" t="s">
@@ -14035,7 +14057,7 @@
       <c r="I29" s="26">
         <v>6.2807941809932109</v>
       </c>
-      <c r="J29" s="36"/>
+      <c r="J29" s="37"/>
     </row>
     <row r="30" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A30" s="25" t="s">
@@ -14065,7 +14087,7 @@
       <c r="I30" s="26">
         <v>6.3671513082216116</v>
       </c>
-      <c r="J30" s="36"/>
+      <c r="J30" s="37"/>
     </row>
     <row r="31" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A31" s="25" t="s">
@@ -14095,7 +14117,7 @@
       <c r="I31" s="26">
         <v>6.4447194345643872</v>
       </c>
-      <c r="J31" s="36"/>
+      <c r="J31" s="37"/>
     </row>
     <row r="32" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A32" s="25" t="s">
@@ -14125,7 +14147,7 @@
       <c r="I32" s="26">
         <v>6.3597316472391725</v>
       </c>
-      <c r="J32" s="36"/>
+      <c r="J32" s="37"/>
     </row>
     <row r="33" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A33" s="25" t="s">
@@ -14155,7 +14177,7 @@
       <c r="I33" s="26">
         <v>6.2245584712274056</v>
       </c>
-      <c r="J33" s="36"/>
+      <c r="J33" s="37"/>
     </row>
     <row r="34" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A34" s="23" t="s">
@@ -14185,7 +14207,7 @@
       <c r="I34" s="24">
         <v>6.2256455918116629</v>
       </c>
-      <c r="J34" s="37"/>
+      <c r="J34" s="38"/>
     </row>
   </sheetData>
   <mergeCells count="3">
@@ -14265,7 +14287,7 @@
       <c r="H2" s="26">
         <v>9.2513300410706787</v>
       </c>
-      <c r="I2" s="38" t="s">
+      <c r="I2" s="39" t="s">
         <v>80</v>
       </c>
       <c r="J2" s="22"/>
@@ -14301,7 +14323,7 @@
       <c r="H3" s="26">
         <v>9.2727881160154872</v>
       </c>
-      <c r="I3" s="38"/>
+      <c r="I3" s="39"/>
     </row>
     <row r="4" spans="1:33" x14ac:dyDescent="0.3">
       <c r="A4" s="25" t="s">
@@ -14328,7 +14350,7 @@
       <c r="H4" s="26">
         <v>9.2888333432264734</v>
       </c>
-      <c r="I4" s="38"/>
+      <c r="I4" s="39"/>
       <c r="Y4" s="22"/>
       <c r="Z4" s="22"/>
       <c r="AA4" s="22"/>
@@ -14364,7 +14386,7 @@
       <c r="H5" s="26">
         <v>9.3336826530210324</v>
       </c>
-      <c r="I5" s="38"/>
+      <c r="I5" s="39"/>
       <c r="Y5" s="22"/>
       <c r="Z5" s="22"/>
       <c r="AA5" s="22"/>
@@ -14400,7 +14422,7 @@
       <c r="H6" s="26">
         <v>9.3949251588094622</v>
       </c>
-      <c r="I6" s="38"/>
+      <c r="I6" s="39"/>
       <c r="Y6" s="22"/>
       <c r="Z6" s="22"/>
       <c r="AA6" s="22"/>
@@ -14436,7 +14458,7 @@
       <c r="H7" s="26">
         <v>9.4386532358591584</v>
       </c>
-      <c r="I7" s="38"/>
+      <c r="I7" s="39"/>
     </row>
     <row r="8" spans="1:33" x14ac:dyDescent="0.3">
       <c r="A8" s="25" t="s">
@@ -14463,7 +14485,7 @@
       <c r="H8" s="26">
         <v>9.4652479928370887</v>
       </c>
-      <c r="I8" s="38"/>
+      <c r="I8" s="39"/>
     </row>
     <row r="9" spans="1:33" x14ac:dyDescent="0.3">
       <c r="A9" s="25" t="s">
@@ -14490,7 +14512,7 @@
       <c r="H9" s="26">
         <v>9.4775097499484104</v>
       </c>
-      <c r="I9" s="38"/>
+      <c r="I9" s="39"/>
     </row>
     <row r="10" spans="1:33" x14ac:dyDescent="0.3">
       <c r="A10" s="25" t="s">
@@ -14517,7 +14539,7 @@
       <c r="H10" s="26">
         <v>9.4829225976822347</v>
       </c>
-      <c r="I10" s="38"/>
+      <c r="I10" s="39"/>
     </row>
     <row r="11" spans="1:33" x14ac:dyDescent="0.3">
       <c r="A11" s="25" t="s">
@@ -14544,7 +14566,7 @@
       <c r="H11" s="26">
         <v>9.4813374065601863</v>
       </c>
-      <c r="I11" s="38"/>
+      <c r="I11" s="39"/>
     </row>
     <row r="12" spans="1:33" x14ac:dyDescent="0.3">
       <c r="A12" s="23" t="s">
@@ -14571,7 +14593,7 @@
       <c r="H12" s="24">
         <v>9.4783533106341995</v>
       </c>
-      <c r="I12" s="39"/>
+      <c r="I12" s="40"/>
     </row>
     <row r="13" spans="1:33" x14ac:dyDescent="0.3">
       <c r="A13" s="27" t="s">
@@ -14598,7 +14620,7 @@
       <c r="H13" s="28">
         <v>8.3206843569337785</v>
       </c>
-      <c r="I13" s="40" t="s">
+      <c r="I13" s="41" t="s">
         <v>81</v>
       </c>
       <c r="J13" s="22"/>
@@ -14634,7 +14656,7 @@
       <c r="H14" s="26">
         <v>8.3210983486660606</v>
       </c>
-      <c r="I14" s="38"/>
+      <c r="I14" s="39"/>
     </row>
     <row r="15" spans="1:33" x14ac:dyDescent="0.3">
       <c r="A15" s="25" t="s">
@@ -14661,7 +14683,7 @@
       <c r="H15" s="26">
         <v>8.3997050288332584</v>
       </c>
-      <c r="I15" s="38"/>
+      <c r="I15" s="39"/>
     </row>
     <row r="16" spans="1:33" x14ac:dyDescent="0.3">
       <c r="A16" s="25" t="s">
@@ -14688,7 +14710,7 @@
       <c r="H16" s="26">
         <v>8.3416944373471313</v>
       </c>
-      <c r="I16" s="38"/>
+      <c r="I16" s="39"/>
     </row>
     <row r="17" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A17" s="25" t="s">
@@ -14715,7 +14737,7 @@
       <c r="H17" s="26">
         <v>8.3169066823766986</v>
       </c>
-      <c r="I17" s="38"/>
+      <c r="I17" s="39"/>
     </row>
     <row r="18" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A18" s="25" t="s">
@@ -14742,7 +14764,7 @@
       <c r="H18" s="26">
         <v>8.3324313723373038</v>
       </c>
-      <c r="I18" s="38"/>
+      <c r="I18" s="39"/>
     </row>
     <row r="19" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A19" s="25" t="s">
@@ -14769,7 +14791,7 @@
       <c r="H19" s="26">
         <v>8.4129527642663078</v>
       </c>
-      <c r="I19" s="38"/>
+      <c r="I19" s="39"/>
     </row>
     <row r="20" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A20" s="25" t="s">
@@ -14796,7 +14818,7 @@
       <c r="H20" s="26">
         <v>8.4946643824256256</v>
       </c>
-      <c r="I20" s="38"/>
+      <c r="I20" s="39"/>
     </row>
     <row r="21" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A21" s="25" t="s">
@@ -14823,7 +14845,7 @@
       <c r="H21" s="26">
         <v>8.3997050288332584</v>
       </c>
-      <c r="I21" s="38"/>
+      <c r="I21" s="39"/>
     </row>
     <row r="22" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A22" s="25" t="s">
@@ -14850,7 +14872,7 @@
       <c r="H22" s="26">
         <v>8.253307202504752</v>
       </c>
-      <c r="I22" s="38"/>
+      <c r="I22" s="39"/>
     </row>
     <row r="23" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A23" s="23" t="s">
@@ -14877,7 +14899,7 @@
       <c r="H23" s="24">
         <v>8.2539799390697119</v>
       </c>
-      <c r="I23" s="39"/>
+      <c r="I23" s="40"/>
     </row>
     <row r="24" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A24" s="27" t="s">
@@ -14904,7 +14926,7 @@
       <c r="H24" s="28">
         <v>9.3551899830134921</v>
       </c>
-      <c r="I24" s="35" t="s">
+      <c r="I24" s="36" t="s">
         <v>82</v>
       </c>
       <c r="J24" s="22"/>
@@ -14940,7 +14962,7 @@
       <c r="H25" s="26">
         <v>9.3777056957348073</v>
       </c>
-      <c r="I25" s="36"/>
+      <c r="I25" s="37"/>
     </row>
     <row r="26" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A26" s="25" t="s">
@@ -14967,7 +14989,7 @@
       <c r="H26" s="26">
         <v>9.4723156752426938</v>
       </c>
-      <c r="I26" s="36"/>
+      <c r="I26" s="37"/>
     </row>
     <row r="27" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A27" s="25" t="s">
@@ -14994,7 +15016,7 @@
       <c r="H27" s="26">
         <v>9.4582602133153362</v>
       </c>
-      <c r="I27" s="36"/>
+      <c r="I27" s="37"/>
     </row>
     <row r="28" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A28" s="25" t="s">
@@ -15021,7 +15043,7 @@
       <c r="H28" s="26">
         <v>9.4931271421144849</v>
       </c>
-      <c r="I28" s="36"/>
+      <c r="I28" s="37"/>
       <c r="J28" s="21"/>
     </row>
     <row r="29" spans="1:16" x14ac:dyDescent="0.3">
@@ -15049,7 +15071,7 @@
       <c r="H29" s="26">
         <v>9.5510599947217294</v>
       </c>
-      <c r="I29" s="36"/>
+      <c r="I29" s="37"/>
       <c r="J29" s="21"/>
       <c r="K29" s="21"/>
       <c r="L29" s="21"/>
@@ -15080,7 +15102,7 @@
       <c r="H30" s="26">
         <v>9.6562582805678048</v>
       </c>
-      <c r="I30" s="36"/>
+      <c r="I30" s="37"/>
       <c r="J30" s="21"/>
     </row>
     <row r="31" spans="1:16" x14ac:dyDescent="0.3">
@@ -15108,7 +15130,7 @@
       <c r="H31" s="26">
         <v>9.747806494192</v>
       </c>
-      <c r="I31" s="36"/>
+      <c r="I31" s="37"/>
       <c r="J31" s="21"/>
     </row>
     <row r="32" spans="1:16" x14ac:dyDescent="0.3">
@@ -15136,7 +15158,7 @@
       <c r="H32" s="26">
         <v>9.6522731177473311</v>
       </c>
-      <c r="I32" s="36"/>
+      <c r="I32" s="37"/>
       <c r="J32" s="21"/>
     </row>
     <row r="33" spans="1:10" x14ac:dyDescent="0.3">
@@ -15164,7 +15186,7 @@
       <c r="H33" s="26">
         <v>9.497746203493767</v>
       </c>
-      <c r="I33" s="36"/>
+      <c r="I33" s="37"/>
       <c r="J33" s="21"/>
     </row>
     <row r="34" spans="1:10" x14ac:dyDescent="0.3">
@@ -15192,7 +15214,7 @@
       <c r="H34" s="24">
         <v>9.4982302441665372</v>
       </c>
-      <c r="I34" s="37"/>
+      <c r="I34" s="38"/>
       <c r="J34" s="21"/>
     </row>
     <row r="35" spans="1:10" x14ac:dyDescent="0.3">

</xml_diff>